<commit_message>
doc: add WKO references as separate columns to Spaltenanalyse_Lieferantenabfrage.xlsx
</commit_message>
<xml_diff>
--- a/Spaltenanalyse_Lieferantenabfrage.xlsx
+++ b/Spaltenanalyse_Lieferantenabfrage.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,8 +46,14 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -64,6 +70,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00EDF2F7"/>
         <bgColor rgb="00EDF2F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A365D"/>
+        <bgColor rgb="001A365D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002C5282"/>
+        <bgColor rgb="002C5282"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,12 +116,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -113,6 +137,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -478,11 +506,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -492,473 +522,658 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Spalte 1: EAN / GTIN (Barcode)</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n"/>
-    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SBS-Analysefeld</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>SBS-Wert / Begründung</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>WKO-Referenz (Kapitel)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Gesetzestext / Zitat</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1"/>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
+          <t>Spalte 1: EAN / GTIN (Barcode)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
           <t>Status:</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Zwingend erforderlich</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Nicht in WKO-Richtlinie</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Die WKO-Richtlinie nennt keine EAN-Pflicht. Dies ist ein rein technischer Schlüssel, der für den Datenbank-Import im Online-Shop zwingend benötigt wird.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Die EAN ist der einzige weltweit eindeutige Schlüssel. Ohne EAN können wir die gelieferten Garantiedaten in Magento nicht automatisch dem richtigen Produkt zuordnen.</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Aufwand für Lieferant:</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Sehr gering, da jeder Hersteller die EANs seiner Produkte im System hat.</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Unbedingt behalten (Hauptschlüssel für Import-Automatisierung).</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="15" customHeight="1"/>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Spalte 2: Lieferanten-Artikelnummer (Herstellernummer)</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n"/>
-    </row>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+    </row>
+    <row r="9" ht="24" customHeight="1"/>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>Spalte 2: Lieferanten-Artikelnummer (Herstellernummer)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
           <t>Status:</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Zwingend erforderlich</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Nicht in WKO-Richtlinie</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Für das Label gesetzlich nicht vorgeschrieben. Dient als organisatorischer Abgleichschlüssel zwischen SBS und dem Lieferanten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>B2B-Systeme arbeiten primär mit Artikelnummern. Falls eine EAN falsch eingetippt wird oder fehlt, ist dies unser einziger Ersatz-Schlüssel zur Zuordnung.</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Aufwand für Lieferant:</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Sehr gering (ist deren eigene interne Nummer).</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="9" t="n"/>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Unbedingt behalten (wichtig für die Kommunikation mit dem Lieferanten).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1"/>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Spalte 3: Marke / Brand</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Unbedingt behalten (wichtig für die Kommunikation mit dem Lieferanten bei Rückfragen).</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="9" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1"/>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>Spalte 3: Marke / Brand</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
           <t>Status:</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Gesetzlich zwingend</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Haltbarkeitsgarantie – was muss mitgeteilt werden?</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Angepasst werden muss:
+'Brand/Trademark' → wird ersetzt durch den Herstellernamen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Entspricht dem editierbaren Feld 'Brand/Trademark' auf dem EU-Garantielabel. Der Lieferant muss eintragen, welcher Markenname dort aufgedruckt werden soll.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Entspricht dem Pflichtfeld 'Brand/Trademark' auf dem EU-Garantielabel und muss dort exakt aufgedruckt werden.</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="n"/>
+      <c r="D18" s="9" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Aufwand für Lieferant:</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Extrem gering.</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="C19" s="9" t="n"/>
+      <c r="D19" s="9" t="n"/>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Unbedingt behalten.</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="15" customHeight="1"/>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Spalte 4: Modellkennung / Model identifier</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="n"/>
-    </row>
+      <c r="C20" s="9" t="n"/>
+      <c r="D20" s="9" t="n"/>
+    </row>
+    <row r="21" ht="24" customHeight="1"/>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
+          <t>Spalte 4: Modellkennung / Model identifier</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
           <t>Status:</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Gesetzlich zwingend</t>
         </is>
       </c>
-    </row>
-    <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Haltbarkeitsgarantie – was muss mitgeteilt werden?</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Angepasst werden muss:
+'Model identifier' → durch die Modellbezeichnung des Produkts</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Entspricht dem editierbaren Feld 'Modellkennung' auf dem EU-Garantielabel. Der Lieferant muss hier die spezifische Modellkennung eintragen, die für dieses Produkt gilt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Entspricht dem Pflichtfeld 'Model identifier' auf dem EU-Garantielabel und muss dort exakt aufgedruckt werden.</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="n"/>
+      <c r="D24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Aufwand für Lieferant:</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Sehr gering.</t>
         </is>
       </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="C25" s="9" t="n"/>
+      <c r="D25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>Unbedingt behalten.</t>
         </is>
       </c>
-    </row>
-    <row r="26" ht="15" customHeight="1"/>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Spalte 5: Artikelbezeichnung</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="n"/>
-    </row>
+      <c r="C26" s="9" t="n"/>
+      <c r="D26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="24" customHeight="1"/>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
+          <t>Spalte 5: Artikelbezeichnung</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n"/>
+      <c r="C28" s="5" t="n"/>
+      <c r="D28" s="5" t="n"/>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
           <t>Status:</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>Verzichtbar (Optional)</t>
         </is>
       </c>
-    </row>
-    <row r="29" ht="40" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Nicht in WKO-Richtlinie</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Für das Label gesetzlich nicht erforderlich (dort stehen nur Marke und Modellkennung).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>Dient nur der manuellen Qualitätskontrolle beim Import. Wird nicht in Magento importiert, da wir eigene Bezeichnungen nutzen.</t>
         </is>
       </c>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="C30" s="9" t="n"/>
+      <c r="D30" s="9" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>Aufwand für Lieferant:</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>Höher (längerer Text zum Eintippen).</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="C31" s="9" t="n"/>
+      <c r="D31" s="9" t="n"/>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>Kann weggelassen werden (reduziert den Aufwand für den Lieferanten).</t>
         </is>
       </c>
-    </row>
-    <row r="32" ht="15" customHeight="1"/>
-    <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Spalte 6: Garantiedauer in Jahren (XX)</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="n"/>
-    </row>
+      <c r="C32" s="9" t="n"/>
+      <c r="D32" s="9" t="n"/>
+    </row>
+    <row r="33" ht="24" customHeight="1"/>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
+          <t>Spalte 6: Garantiedauer in Jahren (XX)</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n"/>
+      <c r="C34" s="5" t="n"/>
+      <c r="D34" s="5" t="n"/>
+    </row>
+    <row r="35" ht="40" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
           <t>Status:</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>Gesetzlich zwingend</t>
         </is>
       </c>
-    </row>
-    <row r="35" ht="40" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Haltbarkeitsgarantie – was muss mitgeteilt werden?</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Angepasst werden muss:
+'XX' → wird ersetzt durch die Anzahl der Garantie-Jahre</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B36" s="7" t="inlineStr">
         <is>
           <t>Entspricht dem editierbaren Feld 'XX' auf dem EU-Garantielabel. Bestimmt den Wert der Garantiejahre auf dem Etikett.</t>
         </is>
       </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="C36" s="9" t="n"/>
+      <c r="D36" s="9" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>Aufwand für Lieferant:</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>Sehr gering (Eingabe einer Ganzzahl &gt; 2).</t>
         </is>
       </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="C37" s="9" t="n"/>
+      <c r="D37" s="9" t="n"/>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>Unbedingt behalten.</t>
         </is>
       </c>
-    </row>
-    <row r="38" ht="15" customHeight="1"/>
-    <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Spalte 7: Link zu den Garantiebedingungen</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="n"/>
-    </row>
+      <c r="C38" s="9" t="n"/>
+      <c r="D38" s="9" t="n"/>
+    </row>
+    <row r="39" ht="24" customHeight="1"/>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
+          <t>Spalte 7: Link zu den Garantiebedingungen</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n"/>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="5" t="n"/>
+    </row>
+    <row r="41" ht="40" customHeight="1">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
           <t>Status:</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>Gesetzlich zwingend</t>
         </is>
       </c>
-    </row>
-    <row r="41" ht="40" customHeight="1">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Technische und grafische Anforderungen</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>QR-Code: Dieser führt Verbraucher zu einer EU-weit einheitlichen Informationsseite mit konkreten Rechten und weiterführenden Details. (Händler-Informationspflicht der Bedingungen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>Gesetzliche Pflicht zur Bereitstellung der Garantieerklärung für den Endkunden. Wird im Shop verlinkt (bzw. für Globus in m.PIM hochgeladen).</t>
         </is>
       </c>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="4" t="inlineStr">
+      <c r="C42" s="9" t="n"/>
+      <c r="D42" s="9" t="n"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>Aufwand für Lieferant:</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B43" s="7" t="inlineStr">
         <is>
           <t>Gering (Eingabe einer Web-URL oder Zusendung als PDF).</t>
         </is>
       </c>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="4" t="inlineStr">
+      <c r="C43" s="9" t="n"/>
+      <c r="D43" s="9" t="n"/>
+    </row>
+    <row r="44" ht="15" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B44" s="7" t="inlineStr">
         <is>
           <t>Unbedingt behalten.</t>
         </is>
       </c>
-    </row>
-    <row r="44" ht="15" customHeight="1"/>
-    <row r="45" ht="24" customHeight="1">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Spalte 8: Bestätigung 'Kostenlose Vollgarantie' (Ja/Nein)</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="n"/>
-    </row>
+      <c r="C44" s="9" t="n"/>
+      <c r="D44" s="9" t="n"/>
+    </row>
+    <row r="45" ht="24" customHeight="1"/>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
+          <t>Spalte 8: Bestätigung 'Kostenlose Vollgarantie' (Ja/Nein)</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n"/>
+      <c r="C46" s="5" t="n"/>
+      <c r="D46" s="5" t="n"/>
+    </row>
+    <row r="47" ht="40" customHeight="1">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
           <t>Status:</t>
         </is>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>Dringend empfohlen zur Risiko-Vermeidung</t>
         </is>
       </c>
-    </row>
-    <row r="47" ht="40" customHeight="1">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Haltbarkeitsgarantie – was muss mitgeteilt werden?</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Wenn ein Hersteller dem Verbraucher eine kostenlose gewerbliche Haltbarkeitsgarantie für die gesamte Ware (d.h. also nicht nur für bestimmte Bestandteile oder Aspekte der Ware) mit einer Dauer von mehr als 2 Jahren gewährt...</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B48" s="7" t="inlineStr">
         <is>
           <t>Das EU-Label darf nur für kostenlose Vollgarantien genutzt werden. Eine Falschanzeige bei Teilgarantien führt zur sofortigen Abmahnbarkeit. Die Bestätigung dient uns als Haftungsnachweis.</t>
         </is>
       </c>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="C48" s="9" t="n"/>
+      <c r="D48" s="9" t="n"/>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t>Aufwand für Lieferant:</t>
         </is>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>Sehr gering (Dropdown-Auswahl Ja/Nein).</t>
         </is>
       </c>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="C49" s="9" t="n"/>
+      <c r="D49" s="9" t="n"/>
+    </row>
+    <row r="50" ht="15" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
         </is>
       </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B50" s="7" t="inlineStr">
         <is>
           <t>Unbedingt behalten.</t>
         </is>
       </c>
-    </row>
-    <row r="50" ht="15" customHeight="1"/>
+      <c r="C50" s="9" t="n"/>
+      <c r="D50" s="9" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A39:B39"/>
+  <mergeCells count="25">
+    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="D34:D37"/>
+    <mergeCell ref="D46:D49"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="D40:D43"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="C16:C19"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="D16:D19"/>
+    <mergeCell ref="C40:C43"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="D28:D31"/>
+    <mergeCell ref="D4:D7"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="C28:C31"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="D10:D13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
doc: fix openpyxl merge bug in Spaltenanalyse_Lieferantenabfrage.xlsx
</commit_message>
<xml_diff>
--- a/Spaltenanalyse_Lieferantenabfrage.xlsx
+++ b/Spaltenanalyse_Lieferantenabfrage.xlsx
@@ -34,6 +34,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="001A365D"/>
       <sz val="11"/>
     </font>
@@ -44,12 +50,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -68,12 +68,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDF2F7"/>
-        <bgColor rgb="00EDF2F7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="001A365D"/>
         <bgColor rgb="001A365D"/>
       </patternFill>
@@ -84,19 +78,20 @@
         <bgColor rgb="002C5282"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF2F7"/>
+        <bgColor rgb="00EDF2F7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <bottom style="thin">
-        <color rgb="00CBD5E0"/>
-      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -116,31 +111,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -544,8 +538,8 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1"/>
-    <row r="4" ht="20" customHeight="1">
+    <row r="3" ht="10" customHeight="1"/>
+    <row r="4" ht="24" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Spalte 1: EAN / GTIN (Barcode)</t>
@@ -555,7 +549,7 @@
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="5" t="n"/>
     </row>
-    <row r="5" ht="40" customHeight="1">
+    <row r="5" ht="20" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Status:</t>
@@ -577,7 +571,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
+    <row r="6" ht="40" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
@@ -588,8 +582,8 @@
           <t>Die EAN ist der einzige weltweit eindeutige Schlüssel. Ohne EAN können wir die gelieferten Garantiedaten in Magento nicht automatisch dem richtigen Produkt zuordnen.</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -602,10 +596,10 @@
           <t>Sehr gering, da jeder Hersteller die EANs seiner Produkte im System hat.</t>
         </is>
       </c>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-    </row>
-    <row r="8" ht="15" customHeight="1">
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
@@ -616,11 +610,11 @@
           <t>Unbedingt behalten (Hauptschlüssel für Import-Automatisierung).</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-    </row>
-    <row r="9" ht="24" customHeight="1"/>
-    <row r="10" ht="20" customHeight="1">
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1"/>
+    <row r="10" ht="24" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Spalte 2: Lieferanten-Artikelnummer (Herstellernummer)</t>
@@ -630,7 +624,7 @@
       <c r="C10" s="5" t="n"/>
       <c r="D10" s="5" t="n"/>
     </row>
-    <row r="11" ht="40" customHeight="1">
+    <row r="11" ht="20" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Status:</t>
@@ -652,7 +646,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
+    <row r="12" ht="40" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
@@ -663,8 +657,8 @@
           <t>B2B-Systeme arbeiten primär mit Artikelnummern. Falls eine EAN falsch eingetippt wird oder fehlt, ist dies unser einziger Ersatz-Schlüssel zur Zuordnung.</t>
         </is>
       </c>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -677,10 +671,10 @@
           <t>Sehr gering (ist deren eigene interne Nummer).</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
-    </row>
-    <row r="14" ht="15" customHeight="1">
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
@@ -691,11 +685,11 @@
           <t>Unbedingt behalten (wichtig für die Kommunikation mit dem Lieferanten bei Rückfragen).</t>
         </is>
       </c>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-    </row>
-    <row r="15" ht="24" customHeight="1"/>
-    <row r="16" ht="20" customHeight="1">
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1"/>
+    <row r="16" ht="24" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Spalte 3: Marke / Brand</t>
@@ -705,7 +699,7 @@
       <c r="C16" s="5" t="n"/>
       <c r="D16" s="5" t="n"/>
     </row>
-    <row r="17" ht="40" customHeight="1">
+    <row r="17" ht="20" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Status:</t>
@@ -728,7 +722,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
+    <row r="18" ht="40" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
@@ -739,8 +733,8 @@
           <t>Entspricht dem Pflichtfeld 'Brand/Trademark' auf dem EU-Garantielabel und muss dort exakt aufgedruckt werden.</t>
         </is>
       </c>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
@@ -753,10 +747,10 @@
           <t>Extrem gering.</t>
         </is>
       </c>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-    </row>
-    <row r="20" ht="15" customHeight="1">
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
@@ -767,11 +761,11 @@
           <t>Unbedingt behalten.</t>
         </is>
       </c>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-    </row>
-    <row r="21" ht="24" customHeight="1"/>
-    <row r="22" ht="20" customHeight="1">
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
+    </row>
+    <row r="21" ht="15" customHeight="1"/>
+    <row r="22" ht="24" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Spalte 4: Modellkennung / Model identifier</t>
@@ -781,7 +775,7 @@
       <c r="C22" s="5" t="n"/>
       <c r="D22" s="5" t="n"/>
     </row>
-    <row r="23" ht="40" customHeight="1">
+    <row r="23" ht="20" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Status:</t>
@@ -804,7 +798,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
+    <row r="24" ht="40" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
@@ -815,8 +809,8 @@
           <t>Entspricht dem Pflichtfeld 'Model identifier' auf dem EU-Garantielabel und muss dort exakt aufgedruckt werden.</t>
         </is>
       </c>
-      <c r="C24" s="9" t="n"/>
-      <c r="D24" s="9" t="n"/>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
@@ -829,10 +823,10 @@
           <t>Sehr gering.</t>
         </is>
       </c>
-      <c r="C25" s="9" t="n"/>
-      <c r="D25" s="9" t="n"/>
-    </row>
-    <row r="26" ht="15" customHeight="1">
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="5" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
@@ -843,11 +837,11 @@
           <t>Unbedingt behalten.</t>
         </is>
       </c>
-      <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
-    </row>
-    <row r="27" ht="24" customHeight="1"/>
-    <row r="28" ht="20" customHeight="1">
+      <c r="C26" s="5" t="n"/>
+      <c r="D26" s="5" t="n"/>
+    </row>
+    <row r="27" ht="15" customHeight="1"/>
+    <row r="28" ht="24" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Spalte 5: Artikelbezeichnung</t>
@@ -857,7 +851,7 @@
       <c r="C28" s="5" t="n"/>
       <c r="D28" s="5" t="n"/>
     </row>
-    <row r="29" ht="40" customHeight="1">
+    <row r="29" ht="20" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Status:</t>
@@ -879,7 +873,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="20" customHeight="1">
+    <row r="30" ht="40" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
@@ -890,8 +884,8 @@
           <t>Dient nur der manuellen Qualitätskontrolle beim Import. Wird nicht in Magento importiert, da wir eigene Bezeichnungen nutzen.</t>
         </is>
       </c>
-      <c r="C30" s="9" t="n"/>
-      <c r="D30" s="9" t="n"/>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
@@ -904,10 +898,10 @@
           <t>Höher (längerer Text zum Eintippen).</t>
         </is>
       </c>
-      <c r="C31" s="9" t="n"/>
-      <c r="D31" s="9" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1">
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
@@ -918,11 +912,11 @@
           <t>Kann weggelassen werden (reduziert den Aufwand für den Lieferanten).</t>
         </is>
       </c>
-      <c r="C32" s="9" t="n"/>
-      <c r="D32" s="9" t="n"/>
-    </row>
-    <row r="33" ht="24" customHeight="1"/>
-    <row r="34" ht="20" customHeight="1">
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="5" t="n"/>
+    </row>
+    <row r="33" ht="15" customHeight="1"/>
+    <row r="34" ht="24" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Spalte 6: Garantiedauer in Jahren (XX)</t>
@@ -932,7 +926,7 @@
       <c r="C34" s="5" t="n"/>
       <c r="D34" s="5" t="n"/>
     </row>
-    <row r="35" ht="40" customHeight="1">
+    <row r="35" ht="20" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Status:</t>
@@ -955,7 +949,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="20" customHeight="1">
+    <row r="36" ht="40" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
@@ -966,8 +960,8 @@
           <t>Entspricht dem editierbaren Feld 'XX' auf dem EU-Garantielabel. Bestimmt den Wert der Garantiejahre auf dem Etikett.</t>
         </is>
       </c>
-      <c r="C36" s="9" t="n"/>
-      <c r="D36" s="9" t="n"/>
+      <c r="C36" s="5" t="n"/>
+      <c r="D36" s="5" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
@@ -980,10 +974,10 @@
           <t>Sehr gering (Eingabe einer Ganzzahl &gt; 2).</t>
         </is>
       </c>
-      <c r="C37" s="9" t="n"/>
-      <c r="D37" s="9" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1">
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="n"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
@@ -994,11 +988,11 @@
           <t>Unbedingt behalten.</t>
         </is>
       </c>
-      <c r="C38" s="9" t="n"/>
-      <c r="D38" s="9" t="n"/>
-    </row>
-    <row r="39" ht="24" customHeight="1"/>
-    <row r="40" ht="20" customHeight="1">
+      <c r="C38" s="5" t="n"/>
+      <c r="D38" s="5" t="n"/>
+    </row>
+    <row r="39" ht="15" customHeight="1"/>
+    <row r="40" ht="24" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Spalte 7: Link zu den Garantiebedingungen</t>
@@ -1008,7 +1002,7 @@
       <c r="C40" s="5" t="n"/>
       <c r="D40" s="5" t="n"/>
     </row>
-    <row r="41" ht="40" customHeight="1">
+    <row r="41" ht="20" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
           <t>Status:</t>
@@ -1030,7 +1024,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="20" customHeight="1">
+    <row r="42" ht="40" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
@@ -1041,8 +1035,8 @@
           <t>Gesetzliche Pflicht zur Bereitstellung der Garantieerklärung für den Endkunden. Wird im Shop verlinkt (bzw. für Globus in m.PIM hochgeladen).</t>
         </is>
       </c>
-      <c r="C42" s="9" t="n"/>
-      <c r="D42" s="9" t="n"/>
+      <c r="C42" s="5" t="n"/>
+      <c r="D42" s="5" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
@@ -1055,10 +1049,10 @@
           <t>Gering (Eingabe einer Web-URL oder Zusendung als PDF).</t>
         </is>
       </c>
-      <c r="C43" s="9" t="n"/>
-      <c r="D43" s="9" t="n"/>
-    </row>
-    <row r="44" ht="15" customHeight="1">
+      <c r="C43" s="5" t="n"/>
+      <c r="D43" s="5" t="n"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
@@ -1069,11 +1063,11 @@
           <t>Unbedingt behalten.</t>
         </is>
       </c>
-      <c r="C44" s="9" t="n"/>
-      <c r="D44" s="9" t="n"/>
-    </row>
-    <row r="45" ht="24" customHeight="1"/>
-    <row r="46" ht="20" customHeight="1">
+      <c r="C44" s="5" t="n"/>
+      <c r="D44" s="5" t="n"/>
+    </row>
+    <row r="45" ht="15" customHeight="1"/>
+    <row r="46" ht="24" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Spalte 8: Bestätigung 'Kostenlose Vollgarantie' (Ja/Nein)</t>
@@ -1083,7 +1077,7 @@
       <c r="C46" s="5" t="n"/>
       <c r="D46" s="5" t="n"/>
     </row>
-    <row r="47" ht="40" customHeight="1">
+    <row r="47" ht="20" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
           <t>Status:</t>
@@ -1105,7 +1099,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="20" customHeight="1">
+    <row r="48" ht="40" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
         <is>
           <t>Nutzen für uns:</t>
@@ -1116,8 +1110,8 @@
           <t>Das EU-Label darf nur für kostenlose Vollgarantien genutzt werden. Eine Falschanzeige bei Teilgarantien führt zur sofortigen Abmahnbarkeit. Die Bestätigung dient uns als Haftungsnachweis.</t>
         </is>
       </c>
-      <c r="C48" s="9" t="n"/>
-      <c r="D48" s="9" t="n"/>
+      <c r="C48" s="5" t="n"/>
+      <c r="D48" s="5" t="n"/>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
@@ -1130,10 +1124,10 @@
           <t>Sehr gering (Dropdown-Auswahl Ja/Nein).</t>
         </is>
       </c>
-      <c r="C49" s="9" t="n"/>
-      <c r="D49" s="9" t="n"/>
-    </row>
-    <row r="50" ht="15" customHeight="1">
+      <c r="C49" s="5" t="n"/>
+      <c r="D49" s="5" t="n"/>
+    </row>
+    <row r="50" ht="20" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
         <is>
           <t>Empfehlung:</t>
@@ -1144,36 +1138,37 @@
           <t>Unbedingt behalten.</t>
         </is>
       </c>
-      <c r="C50" s="9" t="n"/>
-      <c r="D50" s="9" t="n"/>
-    </row>
+      <c r="C50" s="5" t="n"/>
+      <c r="D50" s="5" t="n"/>
+    </row>
+    <row r="51" ht="15" customHeight="1"/>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="D22:D25"/>
-    <mergeCell ref="D34:D37"/>
-    <mergeCell ref="D46:D49"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="D40:D43"/>
-    <mergeCell ref="C4:C7"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="C16:C19"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="D16:D19"/>
-    <mergeCell ref="C40:C43"/>
+    <mergeCell ref="C5:C8"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="C29:C32"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="D11:D14"/>
+    <mergeCell ref="C41:C44"/>
+    <mergeCell ref="C35:C38"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="D17:D20"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="C47:C50"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="D28:D31"/>
-    <mergeCell ref="D4:D7"/>
-    <mergeCell ref="A45:D45"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="C28:C31"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="C34:C37"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="C17:C20"/>
+    <mergeCell ref="D41:D44"/>
+    <mergeCell ref="D47:D50"/>
+    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="C23:C26"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="D5:D8"/>
+    <mergeCell ref="D23:D26"/>
+    <mergeCell ref="D35:D38"/>
+    <mergeCell ref="D29:D32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>